<commit_message>
init: coupang ad dashboard
</commit_message>
<xml_diff>
--- a/RAW/NCA/A01194848_nca_daily_ad_20260601_20260614.xlsx
+++ b/RAW/NCA/A01194848_nca_daily_ad_20260601_20260614.xlsx
@@ -143,10 +143,10 @@
     <t>전체</t>
   </si>
   <si>
-    <t>7.32%</t>
+    <t>1.33%</t>
   </si>
   <si>
-    <t>1.33%</t>
+    <t>7.32%</t>
   </si>
   <si>
     <t>0.84%</t>
@@ -203,13 +203,13 @@
     <t>동영상</t>
   </si>
   <si>
-    <t>36.11%</t>
-  </si>
-  <si>
     <t>0.42%</t>
   </si>
   <si>
     <t>14.01%</t>
+  </si>
+  <si>
+    <t>36.11%</t>
   </si>
   <si>
     <t>1.82%</t>
@@ -224,10 +224,10 @@
     <t>2.94%</t>
   </si>
   <si>
-    <t>30.00%</t>
+    <t>14.61%</t>
   </si>
   <si>
-    <t>14.61%</t>
+    <t>30.00%</t>
   </si>
   <si>
     <t>2.41%</t>
@@ -263,13 +263,13 @@
     <t>1.72%</t>
   </si>
   <si>
+    <t>11.18%</t>
+  </si>
+  <si>
     <t>4.35%</t>
   </si>
   <si>
     <t>30.43%</t>
-  </si>
-  <si>
-    <t>11.18%</t>
   </si>
   <si>
     <t>1.49%</t>
@@ -458,13 +458,13 @@
     <t>20.31%</t>
   </si>
   <si>
-    <t>824.60%</t>
-  </si>
-  <si>
     <t>1.89%</t>
   </si>
   <si>
     <t>1485.59%</t>
+  </si>
+  <si>
+    <t>824.60%</t>
   </si>
   <si>
     <t>5.98%</t>
@@ -686,25 +686,25 @@
     <t>1.47%</t>
   </si>
   <si>
-    <t>35.62%</t>
-  </si>
-  <si>
     <t>0.23%</t>
   </si>
   <si>
     <t>11.06%</t>
   </si>
   <si>
-    <t>1.77%</t>
+    <t>35.62%</t>
   </si>
   <si>
-    <t>18.42%</t>
+    <t>1.77%</t>
   </si>
   <si>
     <t>0.07%</t>
   </si>
   <si>
     <t>9.22%</t>
+  </si>
+  <si>
+    <t>18.42%</t>
   </si>
   <si>
     <t>2.17%</t>
@@ -776,10 +776,10 @@
     <t>2.86%</t>
   </si>
   <si>
-    <t>12.42%</t>
+    <t>38.46%</t>
   </si>
   <si>
-    <t>38.46%</t>
+    <t>12.42%</t>
   </si>
   <si>
     <t>4.76%</t>
@@ -788,13 +788,13 @@
     <t>2.96%</t>
   </si>
   <si>
-    <t>14.29%</t>
-  </si>
-  <si>
     <t>0.60%</t>
   </si>
   <si>
     <t>11.98%</t>
+  </si>
+  <si>
+    <t>14.29%</t>
   </si>
   <si>
     <t>3.98%</t>
@@ -1031,10 +1031,10 @@
     <t>22.58%</t>
   </si>
   <si>
-    <t>0.46%</t>
+    <t>1.15%</t>
   </si>
   <si>
-    <t>1.15%</t>
+    <t>0.46%</t>
   </si>
   <si>
     <t>26.14%</t>
@@ -2051,13 +2051,13 @@
         <v>9.1179241841E10</v>
       </c>
       <c r="O9" t="s" s="0">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="P9" t="n" s="0">
-        <v>41.0</v>
+        <v>75.0</v>
       </c>
       <c r="Q9" t="n" s="0">
-        <v>3.0</v>
+        <v>1.0</v>
       </c>
       <c r="R9" t="s" s="0">
         <v>43</v>
@@ -2066,13 +2066,13 @@
         <v>0.0</v>
       </c>
       <c r="T9" t="n" s="0">
-        <v>3.0</v>
+        <v>1.0</v>
       </c>
       <c r="U9" t="s" s="0">
         <v>43</v>
       </c>
       <c r="V9" t="n" s="0">
-        <v>3952.0</v>
+        <v>168.0</v>
       </c>
       <c r="W9" t="s" s="0">
         <v>31</v>
@@ -2131,13 +2131,13 @@
         <v>9.1179241841E10</v>
       </c>
       <c r="O10" t="s" s="0">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="P10" t="n" s="0">
-        <v>75.0</v>
+        <v>41.0</v>
       </c>
       <c r="Q10" t="n" s="0">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="R10" t="s" s="0">
         <v>44</v>
@@ -2146,13 +2146,13 @@
         <v>0.0</v>
       </c>
       <c r="T10" t="n" s="0">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
       <c r="U10" t="s" s="0">
         <v>44</v>
       </c>
       <c r="V10" t="n" s="0">
-        <v>168.0</v>
+        <v>3952.0</v>
       </c>
       <c r="W10" t="s" s="0">
         <v>31</v>
@@ -2611,28 +2611,28 @@
         <v>9.1179241841E10</v>
       </c>
       <c r="O16" t="s" s="0">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="P16" t="n" s="0">
-        <v>0.0</v>
+        <v>119.0</v>
       </c>
       <c r="Q16" t="n" s="0">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="R16" t="s" s="0">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="S16" t="n" s="0">
         <v>0.0</v>
       </c>
       <c r="T16" t="n" s="0">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="U16" t="s" s="0">
-        <v>31</v>
+        <v>45</v>
       </c>
       <c r="V16" t="n" s="0">
-        <v>0.0</v>
+        <v>882.0</v>
       </c>
       <c r="W16" t="s" s="0">
         <v>31</v>
@@ -2644,7 +2644,7 @@
         <v>0.0</v>
       </c>
       <c r="Z16" t="s" s="0">
-        <v>31</v>
+        <v>39</v>
       </c>
     </row>
     <row r="17">
@@ -2691,28 +2691,28 @@
         <v>9.1179241841E10</v>
       </c>
       <c r="O17" t="s" s="0">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="P17" t="n" s="0">
-        <v>119.0</v>
+        <v>0.0</v>
       </c>
       <c r="Q17" t="n" s="0">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="R17" t="s" s="0">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="S17" t="n" s="0">
         <v>0.0</v>
       </c>
       <c r="T17" t="n" s="0">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="U17" t="s" s="0">
-        <v>45</v>
+        <v>31</v>
       </c>
       <c r="V17" t="n" s="0">
-        <v>882.0</v>
+        <v>0.0</v>
       </c>
       <c r="W17" t="s" s="0">
         <v>31</v>
@@ -2724,7 +2724,7 @@
         <v>0.0</v>
       </c>
       <c r="Z17" t="s" s="0">
-        <v>39</v>
+        <v>31</v>
       </c>
     </row>
     <row r="18">
@@ -3891,13 +3891,13 @@
         <v>9.1179241841E10</v>
       </c>
       <c r="O32" t="s" s="0">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="P32" t="n" s="0">
-        <v>96.0</v>
+        <v>0.0</v>
       </c>
       <c r="Q32" t="n" s="0">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
       <c r="R32" t="s" s="0">
         <v>39</v>
@@ -3906,10 +3906,10 @@
         <v>0.0</v>
       </c>
       <c r="T32" t="n" s="0">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
       <c r="U32" t="s" s="0">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="V32" t="n" s="0">
         <v>0.0</v>
@@ -3971,13 +3971,13 @@
         <v>9.1179241841E10</v>
       </c>
       <c r="O33" t="s" s="0">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="P33" t="n" s="0">
-        <v>0.0</v>
+        <v>96.0</v>
       </c>
       <c r="Q33" t="n" s="0">
-        <v>4.0</v>
+        <v>0.0</v>
       </c>
       <c r="R33" t="s" s="0">
         <v>39</v>
@@ -3986,10 +3986,10 @@
         <v>0.0</v>
       </c>
       <c r="T33" t="n" s="0">
-        <v>4.0</v>
+        <v>0.0</v>
       </c>
       <c r="U33" t="s" s="0">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="V33" t="n" s="0">
         <v>0.0</v>
@@ -4211,28 +4211,28 @@
         <v>9.1179241841E10</v>
       </c>
       <c r="O36" t="s" s="0">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="P36" t="n" s="0">
-        <v>130.0</v>
+        <v>0.0</v>
       </c>
       <c r="Q36" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="R36" t="s" s="0">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="S36" t="n" s="0">
         <v>0.0</v>
       </c>
       <c r="T36" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="U36" t="s" s="0">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="V36" t="n" s="0">
-        <v>1171.0</v>
+        <v>0.0</v>
       </c>
       <c r="W36" t="s" s="0">
         <v>31</v>
@@ -4244,7 +4244,7 @@
         <v>0.0</v>
       </c>
       <c r="Z36" t="s" s="0">
-        <v>39</v>
+        <v>31</v>
       </c>
     </row>
     <row r="37">
@@ -4291,28 +4291,28 @@
         <v>9.1179241841E10</v>
       </c>
       <c r="O37" t="s" s="0">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="P37" t="n" s="0">
-        <v>36.0</v>
+        <v>130.0</v>
       </c>
       <c r="Q37" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="R37" t="s" s="0">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="S37" t="n" s="0">
         <v>0.0</v>
       </c>
       <c r="T37" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="U37" t="s" s="0">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="V37" t="n" s="0">
-        <v>0.0</v>
+        <v>1171.0</v>
       </c>
       <c r="W37" t="s" s="0">
         <v>31</v>
@@ -4324,7 +4324,7 @@
         <v>0.0</v>
       </c>
       <c r="Z37" t="s" s="0">
-        <v>31</v>
+        <v>39</v>
       </c>
     </row>
     <row r="38">
@@ -4371,10 +4371,10 @@
         <v>9.1179241841E10</v>
       </c>
       <c r="O38" t="s" s="0">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="P38" t="n" s="0">
-        <v>0.0</v>
+        <v>36.0</v>
       </c>
       <c r="Q38" t="n" s="0">
         <v>0.0</v>
@@ -4389,7 +4389,7 @@
         <v>0.0</v>
       </c>
       <c r="U38" t="s" s="0">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="V38" t="n" s="0">
         <v>0.0</v>
@@ -4851,10 +4851,10 @@
         <v>9.1179241841E10</v>
       </c>
       <c r="O44" t="s" s="0">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="P44" t="n" s="0">
-        <v>101.0</v>
+        <v>0.0</v>
       </c>
       <c r="Q44" t="n" s="0">
         <v>0.0</v>
@@ -4869,7 +4869,7 @@
         <v>0.0</v>
       </c>
       <c r="U44" t="s" s="0">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="V44" t="n" s="0">
         <v>0.0</v>
@@ -4931,10 +4931,10 @@
         <v>9.1179241841E10</v>
       </c>
       <c r="O45" t="s" s="0">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="P45" t="n" s="0">
-        <v>0.0</v>
+        <v>101.0</v>
       </c>
       <c r="Q45" t="n" s="0">
         <v>0.0</v>
@@ -4949,7 +4949,7 @@
         <v>0.0</v>
       </c>
       <c r="U45" t="s" s="0">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="V45" t="n" s="0">
         <v>0.0</v>
@@ -6131,28 +6131,28 @@
         <v>0.0</v>
       </c>
       <c r="O60" t="s" s="0">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="P60" t="n" s="0">
-        <v>36.0</v>
+        <v>471.0</v>
       </c>
       <c r="Q60" t="n" s="0">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
       <c r="R60" t="s" s="0">
-        <v>39</v>
+        <v>63</v>
       </c>
       <c r="S60" t="n" s="0">
-        <v>14.0</v>
+        <v>66.0</v>
       </c>
       <c r="T60" t="n" s="0">
-        <v>13.0</v>
+        <v>66.0</v>
       </c>
       <c r="U60" t="s" s="0">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="V60" t="n" s="0">
-        <v>71.0</v>
+        <v>2498.0</v>
       </c>
       <c r="W60" t="s" s="0">
         <v>31</v>
@@ -6211,28 +6211,28 @@
         <v>0.0</v>
       </c>
       <c r="O61" t="s" s="0">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="P61" t="n" s="0">
-        <v>471.0</v>
+        <v>36.0</v>
       </c>
       <c r="Q61" t="n" s="0">
-        <v>2.0</v>
+        <v>0.0</v>
       </c>
       <c r="R61" t="s" s="0">
-        <v>64</v>
+        <v>39</v>
       </c>
       <c r="S61" t="n" s="0">
-        <v>66.0</v>
+        <v>14.0</v>
       </c>
       <c r="T61" t="n" s="0">
-        <v>66.0</v>
+        <v>13.0</v>
       </c>
       <c r="U61" t="s" s="0">
         <v>65</v>
       </c>
       <c r="V61" t="n" s="0">
-        <v>2498.0</v>
+        <v>71.0</v>
       </c>
       <c r="W61" t="s" s="0">
         <v>31</v>
@@ -6371,28 +6371,28 @@
         <v>9.0174024543E10</v>
       </c>
       <c r="O63" t="s" s="0">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="P63" t="n" s="0">
-        <v>55.0</v>
+        <v>87.0</v>
       </c>
       <c r="Q63" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="R63" t="s" s="0">
-        <v>66</v>
+        <v>39</v>
       </c>
       <c r="S63" t="n" s="0">
         <v>0.0</v>
       </c>
       <c r="T63" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="U63" t="s" s="0">
-        <v>66</v>
+        <v>39</v>
       </c>
       <c r="V63" t="n" s="0">
-        <v>4553.0</v>
+        <v>0.0</v>
       </c>
       <c r="W63" t="s" s="0">
         <v>31</v>
@@ -6404,7 +6404,7 @@
         <v>0.0</v>
       </c>
       <c r="Z63" t="s" s="0">
-        <v>39</v>
+        <v>31</v>
       </c>
     </row>
     <row r="64">
@@ -6451,28 +6451,28 @@
         <v>9.0174024543E10</v>
       </c>
       <c r="O64" t="s" s="0">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="P64" t="n" s="0">
-        <v>87.0</v>
+        <v>55.0</v>
       </c>
       <c r="Q64" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="R64" t="s" s="0">
-        <v>39</v>
+        <v>66</v>
       </c>
       <c r="S64" t="n" s="0">
         <v>0.0</v>
       </c>
       <c r="T64" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="U64" t="s" s="0">
-        <v>39</v>
+        <v>66</v>
       </c>
       <c r="V64" t="n" s="0">
-        <v>0.0</v>
+        <v>4553.0</v>
       </c>
       <c r="W64" t="s" s="0">
         <v>31</v>
@@ -6484,7 +6484,7 @@
         <v>0.0</v>
       </c>
       <c r="Z64" t="s" s="0">
-        <v>31</v>
+        <v>39</v>
       </c>
     </row>
     <row r="65">
@@ -7251,10 +7251,10 @@
         <v>0.0</v>
       </c>
       <c r="O74" t="s" s="0">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="P74" t="n" s="0">
-        <v>10.0</v>
+        <v>178.0</v>
       </c>
       <c r="Q74" t="n" s="0">
         <v>0.0</v>
@@ -7263,16 +7263,16 @@
         <v>39</v>
       </c>
       <c r="S74" t="n" s="0">
-        <v>3.0</v>
+        <v>26.0</v>
       </c>
       <c r="T74" t="n" s="0">
-        <v>3.0</v>
+        <v>26.0</v>
       </c>
       <c r="U74" t="s" s="0">
         <v>70</v>
       </c>
       <c r="V74" t="n" s="0">
-        <v>32.0</v>
+        <v>659.0</v>
       </c>
       <c r="W74" t="s" s="0">
         <v>31</v>
@@ -7331,10 +7331,10 @@
         <v>0.0</v>
       </c>
       <c r="O75" t="s" s="0">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="P75" t="n" s="0">
-        <v>178.0</v>
+        <v>10.0</v>
       </c>
       <c r="Q75" t="n" s="0">
         <v>0.0</v>
@@ -7343,16 +7343,16 @@
         <v>39</v>
       </c>
       <c r="S75" t="n" s="0">
-        <v>26.0</v>
+        <v>3.0</v>
       </c>
       <c r="T75" t="n" s="0">
-        <v>26.0</v>
+        <v>3.0</v>
       </c>
       <c r="U75" t="s" s="0">
         <v>71</v>
       </c>
       <c r="V75" t="n" s="0">
-        <v>659.0</v>
+        <v>32.0</v>
       </c>
       <c r="W75" t="s" s="0">
         <v>31</v>
@@ -8931,28 +8931,28 @@
         <v>0.0</v>
       </c>
       <c r="O95" t="s" s="0">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="P95" t="n" s="0">
-        <v>23.0</v>
+        <v>170.0</v>
       </c>
       <c r="Q95" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="R95" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="S95" t="n" s="0">
+        <v>19.0</v>
+      </c>
+      <c r="T95" t="n" s="0">
+        <v>19.0</v>
+      </c>
+      <c r="U95" t="s" s="0">
         <v>83</v>
       </c>
-      <c r="S95" t="n" s="0">
-        <v>7.0</v>
-      </c>
-      <c r="T95" t="n" s="0">
-        <v>7.0</v>
-      </c>
-      <c r="U95" t="s" s="0">
-        <v>84</v>
-      </c>
       <c r="V95" t="n" s="0">
-        <v>53.0</v>
+        <v>657.0</v>
       </c>
       <c r="W95" t="s" s="0">
         <v>31</v>
@@ -9011,28 +9011,28 @@
         <v>0.0</v>
       </c>
       <c r="O96" t="s" s="0">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="P96" t="n" s="0">
-        <v>170.0</v>
+        <v>23.0</v>
       </c>
       <c r="Q96" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="R96" t="s" s="0">
-        <v>39</v>
+        <v>84</v>
       </c>
       <c r="S96" t="n" s="0">
-        <v>19.0</v>
+        <v>7.0</v>
       </c>
       <c r="T96" t="n" s="0">
-        <v>19.0</v>
+        <v>7.0</v>
       </c>
       <c r="U96" t="s" s="0">
         <v>85</v>
       </c>
       <c r="V96" t="n" s="0">
-        <v>657.0</v>
+        <v>53.0</v>
       </c>
       <c r="W96" t="s" s="0">
         <v>31</v>
@@ -14771,28 +14771,28 @@
         <v>9.3934937349E10</v>
       </c>
       <c r="O168" t="s" s="0">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="P168" t="n" s="0">
-        <v>0.0</v>
+        <v>793.0</v>
       </c>
       <c r="Q168" t="n" s="0">
-        <v>279.0</v>
+        <v>15.0</v>
       </c>
       <c r="R168" t="s" s="0">
-        <v>39</v>
+        <v>148</v>
       </c>
       <c r="S168" t="n" s="0">
         <v>0.0</v>
       </c>
       <c r="T168" t="n" s="0">
-        <v>279.0</v>
+        <v>15.0</v>
       </c>
       <c r="U168" t="s" s="0">
-        <v>31</v>
+        <v>148</v>
       </c>
       <c r="V168" t="n" s="0">
-        <v>3626.0</v>
+        <v>5412.0</v>
       </c>
       <c r="W168" t="s" s="0">
         <v>31</v>
@@ -14801,10 +14801,10 @@
         <v>38</v>
       </c>
       <c r="Y168" t="n" s="0">
-        <v>29900.0</v>
+        <v>80400.0</v>
       </c>
       <c r="Z168" t="s" s="0">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="169">
@@ -14851,28 +14851,28 @@
         <v>9.3934937349E10</v>
       </c>
       <c r="O169" t="s" s="0">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="P169" t="n" s="0">
-        <v>793.0</v>
+        <v>0.0</v>
       </c>
       <c r="Q169" t="n" s="0">
-        <v>15.0</v>
+        <v>279.0</v>
       </c>
       <c r="R169" t="s" s="0">
-        <v>149</v>
+        <v>39</v>
       </c>
       <c r="S169" t="n" s="0">
         <v>0.0</v>
       </c>
       <c r="T169" t="n" s="0">
-        <v>15.0</v>
+        <v>279.0</v>
       </c>
       <c r="U169" t="s" s="0">
-        <v>149</v>
+        <v>31</v>
       </c>
       <c r="V169" t="n" s="0">
-        <v>5412.0</v>
+        <v>3626.0</v>
       </c>
       <c r="W169" t="s" s="0">
         <v>31</v>
@@ -14881,7 +14881,7 @@
         <v>38</v>
       </c>
       <c r="Y169" t="n" s="0">
-        <v>80400.0</v>
+        <v>29900.0</v>
       </c>
       <c r="Z169" t="s" s="0">
         <v>150</v>
@@ -18451,10 +18451,10 @@
         <v>9.2605081605E10</v>
       </c>
       <c r="O214" t="s" s="0">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="P214" t="n" s="0">
-        <v>0.0</v>
+        <v>99.0</v>
       </c>
       <c r="Q214" t="n" s="0">
         <v>0.0</v>
@@ -18469,7 +18469,7 @@
         <v>0.0</v>
       </c>
       <c r="U214" t="s" s="0">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="V214" t="n" s="0">
         <v>0.0</v>
@@ -18531,10 +18531,10 @@
         <v>9.2605081605E10</v>
       </c>
       <c r="O215" t="s" s="0">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="P215" t="n" s="0">
-        <v>99.0</v>
+        <v>0.0</v>
       </c>
       <c r="Q215" t="n" s="0">
         <v>0.0</v>
@@ -18549,7 +18549,7 @@
         <v>0.0</v>
       </c>
       <c r="U215" t="s" s="0">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="V215" t="n" s="0">
         <v>0.0</v>
@@ -19411,28 +19411,28 @@
         <v>9.2605081605E10</v>
       </c>
       <c r="O226" t="s" s="0">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="P226" t="n" s="0">
-        <v>60.0</v>
+        <v>0.0</v>
       </c>
       <c r="Q226" t="n" s="0">
-        <v>2.0</v>
+        <v>0.0</v>
       </c>
       <c r="R226" t="s" s="0">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="S226" t="n" s="0">
         <v>0.0</v>
       </c>
       <c r="T226" t="n" s="0">
-        <v>2.0</v>
+        <v>0.0</v>
       </c>
       <c r="U226" t="s" s="0">
-        <v>60</v>
+        <v>31</v>
       </c>
       <c r="V226" t="n" s="0">
-        <v>1852.0</v>
+        <v>0.0</v>
       </c>
       <c r="W226" t="s" s="0">
         <v>31</v>
@@ -19444,7 +19444,7 @@
         <v>0.0</v>
       </c>
       <c r="Z226" t="s" s="0">
-        <v>39</v>
+        <v>31</v>
       </c>
     </row>
     <row r="227">
@@ -19491,28 +19491,28 @@
         <v>9.2605081605E10</v>
       </c>
       <c r="O227" t="s" s="0">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="P227" t="n" s="0">
-        <v>0.0</v>
+        <v>60.0</v>
       </c>
       <c r="Q227" t="n" s="0">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
       <c r="R227" t="s" s="0">
-        <v>39</v>
+        <v>60</v>
       </c>
       <c r="S227" t="n" s="0">
         <v>0.0</v>
       </c>
       <c r="T227" t="n" s="0">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
       <c r="U227" t="s" s="0">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="V227" t="n" s="0">
-        <v>0.0</v>
+        <v>1852.0</v>
       </c>
       <c r="W227" t="s" s="0">
         <v>31</v>
@@ -19524,7 +19524,7 @@
         <v>0.0</v>
       </c>
       <c r="Z227" t="s" s="0">
-        <v>31</v>
+        <v>39</v>
       </c>
     </row>
     <row r="228">
@@ -23091,28 +23091,28 @@
         <v>9.2605020671E10</v>
       </c>
       <c r="O272" t="s" s="0">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="P272" t="n" s="0">
-        <v>25.0</v>
+        <v>71.0</v>
       </c>
       <c r="Q272" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="R272" t="s" s="0">
-        <v>39</v>
+        <v>212</v>
       </c>
       <c r="S272" t="n" s="0">
         <v>0.0</v>
       </c>
       <c r="T272" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="U272" t="s" s="0">
-        <v>39</v>
+        <v>212</v>
       </c>
       <c r="V272" t="n" s="0">
-        <v>0.0</v>
+        <v>468.0</v>
       </c>
       <c r="W272" t="s" s="0">
         <v>31</v>
@@ -23124,7 +23124,7 @@
         <v>0.0</v>
       </c>
       <c r="Z272" t="s" s="0">
-        <v>31</v>
+        <v>39</v>
       </c>
     </row>
     <row r="273">
@@ -23171,28 +23171,28 @@
         <v>9.2605020671E10</v>
       </c>
       <c r="O273" t="s" s="0">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="P273" t="n" s="0">
-        <v>71.0</v>
+        <v>25.0</v>
       </c>
       <c r="Q273" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="R273" t="s" s="0">
-        <v>212</v>
+        <v>39</v>
       </c>
       <c r="S273" t="n" s="0">
         <v>0.0</v>
       </c>
       <c r="T273" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="U273" t="s" s="0">
-        <v>212</v>
+        <v>39</v>
       </c>
       <c r="V273" t="n" s="0">
-        <v>468.0</v>
+        <v>0.0</v>
       </c>
       <c r="W273" t="s" s="0">
         <v>31</v>
@@ -23204,7 +23204,7 @@
         <v>0.0</v>
       </c>
       <c r="Z273" t="s" s="0">
-        <v>39</v>
+        <v>31</v>
       </c>
     </row>
     <row r="274">
@@ -23509,7 +23509,7 @@
         <v>6.0</v>
       </c>
       <c r="U277" t="s" s="0">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="V277" t="n" s="0">
         <v>40.0</v>
@@ -24771,28 +24771,28 @@
         <v>9.2605020671E10</v>
       </c>
       <c r="O293" t="s" s="0">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="P293" t="n" s="0">
-        <v>59.0</v>
+        <v>23.0</v>
       </c>
       <c r="Q293" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="R293" t="s" s="0">
-        <v>39</v>
+        <v>84</v>
       </c>
       <c r="S293" t="n" s="0">
         <v>0.0</v>
       </c>
       <c r="T293" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="U293" t="s" s="0">
-        <v>39</v>
+        <v>84</v>
       </c>
       <c r="V293" t="n" s="0">
-        <v>0.0</v>
+        <v>2095.0</v>
       </c>
       <c r="W293" t="s" s="0">
         <v>31</v>
@@ -24804,7 +24804,7 @@
         <v>0.0</v>
       </c>
       <c r="Z293" t="s" s="0">
-        <v>31</v>
+        <v>39</v>
       </c>
     </row>
     <row r="294">
@@ -24851,28 +24851,28 @@
         <v>9.2605020671E10</v>
       </c>
       <c r="O294" t="s" s="0">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="P294" t="n" s="0">
-        <v>23.0</v>
+        <v>59.0</v>
       </c>
       <c r="Q294" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="R294" t="s" s="0">
-        <v>83</v>
+        <v>39</v>
       </c>
       <c r="S294" t="n" s="0">
         <v>0.0</v>
       </c>
       <c r="T294" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="U294" t="s" s="0">
-        <v>83</v>
+        <v>39</v>
       </c>
       <c r="V294" t="n" s="0">
-        <v>2095.0</v>
+        <v>0.0</v>
       </c>
       <c r="W294" t="s" s="0">
         <v>31</v>
@@ -24884,7 +24884,7 @@
         <v>0.0</v>
       </c>
       <c r="Z294" t="s" s="0">
-        <v>39</v>
+        <v>31</v>
       </c>
     </row>
     <row r="295">
@@ -25651,28 +25651,28 @@
         <v>0.0</v>
       </c>
       <c r="O304" t="s" s="0">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="P304" t="n" s="0">
-        <v>73.0</v>
+        <v>443.0</v>
       </c>
       <c r="Q304" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="R304" t="s" s="0">
-        <v>39</v>
+        <v>224</v>
       </c>
       <c r="S304" t="n" s="0">
-        <v>27.0</v>
+        <v>49.0</v>
       </c>
       <c r="T304" t="n" s="0">
-        <v>26.0</v>
+        <v>49.0</v>
       </c>
       <c r="U304" t="s" s="0">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="V304" t="n" s="0">
-        <v>152.0</v>
+        <v>1357.0</v>
       </c>
       <c r="W304" t="s" s="0">
         <v>31</v>
@@ -25731,28 +25731,28 @@
         <v>0.0</v>
       </c>
       <c r="O305" t="s" s="0">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="P305" t="n" s="0">
-        <v>443.0</v>
+        <v>73.0</v>
       </c>
       <c r="Q305" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="R305" t="s" s="0">
-        <v>225</v>
+        <v>39</v>
       </c>
       <c r="S305" t="n" s="0">
-        <v>49.0</v>
+        <v>27.0</v>
       </c>
       <c r="T305" t="n" s="0">
-        <v>49.0</v>
+        <v>26.0</v>
       </c>
       <c r="U305" t="s" s="0">
         <v>226</v>
       </c>
       <c r="V305" t="n" s="0">
-        <v>1357.0</v>
+        <v>152.0</v>
       </c>
       <c r="W305" t="s" s="0">
         <v>31</v>
@@ -26060,7 +26060,7 @@
         <v>1.0</v>
       </c>
       <c r="R309" t="s" s="0">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="S309" t="n" s="0">
         <v>0.0</v>
@@ -26069,7 +26069,7 @@
         <v>1.0</v>
       </c>
       <c r="U309" t="s" s="0">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="V309" t="n" s="0">
         <v>1560.0</v>
@@ -26211,28 +26211,28 @@
         <v>0.0</v>
       </c>
       <c r="O311" t="s" s="0">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="P311" t="n" s="0">
-        <v>38.0</v>
+        <v>1432.0</v>
       </c>
       <c r="Q311" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="R311" t="s" s="0">
-        <v>39</v>
+        <v>228</v>
       </c>
       <c r="S311" t="n" s="0">
-        <v>8.0</v>
+        <v>131.0</v>
       </c>
       <c r="T311" t="n" s="0">
-        <v>7.0</v>
+        <v>132.0</v>
       </c>
       <c r="U311" t="s" s="0">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="V311" t="n" s="0">
-        <v>38.0</v>
+        <v>5459.0</v>
       </c>
       <c r="W311" t="s" s="0">
         <v>31</v>
@@ -26291,28 +26291,28 @@
         <v>0.0</v>
       </c>
       <c r="O312" t="s" s="0">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="P312" t="n" s="0">
-        <v>1432.0</v>
+        <v>38.0</v>
       </c>
       <c r="Q312" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="R312" t="s" s="0">
-        <v>229</v>
+        <v>39</v>
       </c>
       <c r="S312" t="n" s="0">
-        <v>131.0</v>
+        <v>8.0</v>
       </c>
       <c r="T312" t="n" s="0">
-        <v>132.0</v>
+        <v>7.0</v>
       </c>
       <c r="U312" t="s" s="0">
         <v>230</v>
       </c>
       <c r="V312" t="n" s="0">
-        <v>5459.0</v>
+        <v>38.0</v>
       </c>
       <c r="W312" t="s" s="0">
         <v>31</v>
@@ -29571,10 +29571,10 @@
         <v>0.0</v>
       </c>
       <c r="O353" t="s" s="0">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="P353" t="n" s="0">
-        <v>153.0</v>
+        <v>13.0</v>
       </c>
       <c r="Q353" t="n" s="0">
         <v>0.0</v>
@@ -29583,16 +29583,16 @@
         <v>39</v>
       </c>
       <c r="S353" t="n" s="0">
-        <v>19.0</v>
+        <v>5.0</v>
       </c>
       <c r="T353" t="n" s="0">
-        <v>19.0</v>
+        <v>5.0</v>
       </c>
       <c r="U353" t="s" s="0">
         <v>254</v>
       </c>
       <c r="V353" t="n" s="0">
-        <v>616.0</v>
+        <v>31.0</v>
       </c>
       <c r="W353" t="s" s="0">
         <v>31</v>
@@ -29651,10 +29651,10 @@
         <v>0.0</v>
       </c>
       <c r="O354" t="s" s="0">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="P354" t="n" s="0">
-        <v>13.0</v>
+        <v>153.0</v>
       </c>
       <c r="Q354" t="n" s="0">
         <v>0.0</v>
@@ -29663,16 +29663,16 @@
         <v>39</v>
       </c>
       <c r="S354" t="n" s="0">
-        <v>5.0</v>
+        <v>19.0</v>
       </c>
       <c r="T354" t="n" s="0">
-        <v>5.0</v>
+        <v>19.0</v>
       </c>
       <c r="U354" t="s" s="0">
         <v>255</v>
       </c>
       <c r="V354" t="n" s="0">
-        <v>31.0</v>
+        <v>616.0</v>
       </c>
       <c r="W354" t="s" s="0">
         <v>31</v>
@@ -30131,28 +30131,28 @@
         <v>0.0</v>
       </c>
       <c r="O360" t="s" s="0">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="P360" t="n" s="0">
-        <v>21.0</v>
+        <v>167.0</v>
       </c>
       <c r="Q360" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="R360" t="s" s="0">
-        <v>39</v>
+        <v>258</v>
       </c>
       <c r="S360" t="n" s="0">
-        <v>5.0</v>
+        <v>20.0</v>
       </c>
       <c r="T360" t="n" s="0">
-        <v>3.0</v>
+        <v>20.0</v>
       </c>
       <c r="U360" t="s" s="0">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="V360" t="n" s="0">
-        <v>33.0</v>
+        <v>522.0</v>
       </c>
       <c r="W360" t="s" s="0">
         <v>31</v>
@@ -30211,28 +30211,28 @@
         <v>0.0</v>
       </c>
       <c r="O361" t="s" s="0">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="P361" t="n" s="0">
-        <v>167.0</v>
+        <v>21.0</v>
       </c>
       <c r="Q361" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="R361" t="s" s="0">
-        <v>259</v>
+        <v>39</v>
       </c>
       <c r="S361" t="n" s="0">
-        <v>20.0</v>
+        <v>5.0</v>
       </c>
       <c r="T361" t="n" s="0">
-        <v>20.0</v>
+        <v>3.0</v>
       </c>
       <c r="U361" t="s" s="0">
         <v>260</v>
       </c>
       <c r="V361" t="n" s="0">
-        <v>522.0</v>
+        <v>33.0</v>
       </c>
       <c r="W361" t="s" s="0">
         <v>31</v>
@@ -31491,28 +31491,28 @@
         <v>9.200897372E10</v>
       </c>
       <c r="O377" t="s" s="0">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="P377" t="n" s="0">
-        <v>39.0</v>
+        <v>176.0</v>
       </c>
       <c r="Q377" t="n" s="0">
-        <v>2.0</v>
+        <v>7.0</v>
       </c>
       <c r="R377" t="s" s="0">
-        <v>270</v>
+        <v>261</v>
       </c>
       <c r="S377" t="n" s="0">
         <v>0.0</v>
       </c>
       <c r="T377" t="n" s="0">
-        <v>2.0</v>
+        <v>7.0</v>
       </c>
       <c r="U377" t="s" s="0">
-        <v>270</v>
+        <v>261</v>
       </c>
       <c r="V377" t="n" s="0">
-        <v>1434.0</v>
+        <v>2969.0</v>
       </c>
       <c r="W377" t="s" s="0">
         <v>31</v>
@@ -31571,28 +31571,28 @@
         <v>9.200897372E10</v>
       </c>
       <c r="O378" t="s" s="0">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="P378" t="n" s="0">
-        <v>176.0</v>
+        <v>39.0</v>
       </c>
       <c r="Q378" t="n" s="0">
-        <v>7.0</v>
+        <v>2.0</v>
       </c>
       <c r="R378" t="s" s="0">
-        <v>261</v>
+        <v>270</v>
       </c>
       <c r="S378" t="n" s="0">
         <v>0.0</v>
       </c>
       <c r="T378" t="n" s="0">
-        <v>7.0</v>
+        <v>2.0</v>
       </c>
       <c r="U378" t="s" s="0">
-        <v>261</v>
+        <v>270</v>
       </c>
       <c r="V378" t="n" s="0">
-        <v>2969.0</v>
+        <v>1434.0</v>
       </c>
       <c r="W378" t="s" s="0">
         <v>31</v>
@@ -32371,28 +32371,28 @@
         <v>0.0</v>
       </c>
       <c r="O388" t="s" s="0">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="P388" t="n" s="0">
-        <v>2.0</v>
+        <v>182.0</v>
       </c>
       <c r="Q388" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="R388" t="s" s="0">
-        <v>39</v>
+        <v>101</v>
       </c>
       <c r="S388" t="n" s="0">
-        <v>1.0</v>
+        <v>26.0</v>
       </c>
       <c r="T388" t="n" s="0">
-        <v>1.0</v>
+        <v>26.0</v>
       </c>
       <c r="U388" t="s" s="0">
-        <v>274</v>
+        <v>260</v>
       </c>
       <c r="V388" t="n" s="0">
-        <v>15.0</v>
+        <v>530.0</v>
       </c>
       <c r="W388" t="s" s="0">
         <v>31</v>
@@ -32451,28 +32451,28 @@
         <v>0.0</v>
       </c>
       <c r="O389" t="s" s="0">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="P389" t="n" s="0">
-        <v>182.0</v>
+        <v>2.0</v>
       </c>
       <c r="Q389" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="R389" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="S389" t="n" s="0">
         <v>1.0</v>
       </c>
-      <c r="R389" t="s" s="0">
-        <v>101</v>
-      </c>
-      <c r="S389" t="n" s="0">
-        <v>26.0</v>
-      </c>
       <c r="T389" t="n" s="0">
-        <v>26.0</v>
+        <v>1.0</v>
       </c>
       <c r="U389" t="s" s="0">
-        <v>258</v>
+        <v>274</v>
       </c>
       <c r="V389" t="n" s="0">
-        <v>530.0</v>
+        <v>15.0</v>
       </c>
       <c r="W389" t="s" s="0">
         <v>31</v>
@@ -33820,7 +33820,7 @@
         <v>7.0</v>
       </c>
       <c r="R406" t="s" s="0">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="S406" t="n" s="0">
         <v>0.0</v>
@@ -33829,7 +33829,7 @@
         <v>7.0</v>
       </c>
       <c r="U406" t="s" s="0">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="V406" t="n" s="0">
         <v>2625.0</v>
@@ -35651,10 +35651,10 @@
         <v>0.0</v>
       </c>
       <c r="O429" t="s" s="0">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="P429" t="n" s="0">
-        <v>7.0</v>
+        <v>0.0</v>
       </c>
       <c r="Q429" t="n" s="0">
         <v>0.0</v>
@@ -35669,7 +35669,7 @@
         <v>0.0</v>
       </c>
       <c r="U429" t="s" s="0">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="V429" t="n" s="0">
         <v>0.0</v>
@@ -35731,10 +35731,10 @@
         <v>0.0</v>
       </c>
       <c r="O430" t="s" s="0">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="P430" t="n" s="0">
-        <v>0.0</v>
+        <v>7.0</v>
       </c>
       <c r="Q430" t="n" s="0">
         <v>0.0</v>
@@ -35749,7 +35749,7 @@
         <v>0.0</v>
       </c>
       <c r="U430" t="s" s="0">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="V430" t="n" s="0">
         <v>0.0</v>
@@ -45651,13 +45651,13 @@
         <v>9.0174073185E10</v>
       </c>
       <c r="O554" t="s" s="0">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="P554" t="n" s="0">
-        <v>437.0</v>
+        <v>87.0</v>
       </c>
       <c r="Q554" t="n" s="0">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="R554" t="s" s="0">
         <v>339</v>
@@ -45666,13 +45666,13 @@
         <v>0.0</v>
       </c>
       <c r="T554" t="n" s="0">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="U554" t="s" s="0">
         <v>339</v>
       </c>
       <c r="V554" t="n" s="0">
-        <v>524.0</v>
+        <v>1905.0</v>
       </c>
       <c r="W554" t="s" s="0">
         <v>31</v>
@@ -45731,13 +45731,13 @@
         <v>9.0174073185E10</v>
       </c>
       <c r="O555" t="s" s="0">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="P555" t="n" s="0">
-        <v>87.0</v>
+        <v>437.0</v>
       </c>
       <c r="Q555" t="n" s="0">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="R555" t="s" s="0">
         <v>340</v>
@@ -45746,13 +45746,13 @@
         <v>0.0</v>
       </c>
       <c r="T555" t="n" s="0">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="U555" t="s" s="0">
         <v>340</v>
       </c>
       <c r="V555" t="n" s="0">
-        <v>1905.0</v>
+        <v>524.0</v>
       </c>
       <c r="W555" t="s" s="0">
         <v>31</v>
@@ -46211,28 +46211,28 @@
         <v>9.0174073185E10</v>
       </c>
       <c r="O561" t="s" s="0">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="P561" t="n" s="0">
-        <v>79.0</v>
+        <v>554.0</v>
       </c>
       <c r="Q561" t="n" s="0">
-        <v>4.0</v>
+        <v>8.0</v>
       </c>
       <c r="R561" t="s" s="0">
-        <v>343</v>
+        <v>115</v>
       </c>
       <c r="S561" t="n" s="0">
         <v>0.0</v>
       </c>
       <c r="T561" t="n" s="0">
-        <v>4.0</v>
+        <v>8.0</v>
       </c>
       <c r="U561" t="s" s="0">
-        <v>343</v>
+        <v>115</v>
       </c>
       <c r="V561" t="n" s="0">
-        <v>5557.0</v>
+        <v>5190.0</v>
       </c>
       <c r="W561" t="s" s="0">
         <v>31</v>
@@ -46291,28 +46291,28 @@
         <v>9.0174073185E10</v>
       </c>
       <c r="O562" t="s" s="0">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="P562" t="n" s="0">
-        <v>554.0</v>
+        <v>79.0</v>
       </c>
       <c r="Q562" t="n" s="0">
-        <v>8.0</v>
+        <v>4.0</v>
       </c>
       <c r="R562" t="s" s="0">
-        <v>115</v>
+        <v>343</v>
       </c>
       <c r="S562" t="n" s="0">
         <v>0.0</v>
       </c>
       <c r="T562" t="n" s="0">
-        <v>8.0</v>
+        <v>4.0</v>
       </c>
       <c r="U562" t="s" s="0">
-        <v>115</v>
+        <v>343</v>
       </c>
       <c r="V562" t="n" s="0">
-        <v>5190.0</v>
+        <v>5557.0</v>
       </c>
       <c r="W562" t="s" s="0">
         <v>31</v>
@@ -47891,28 +47891,28 @@
         <v>9.0174073185E10</v>
       </c>
       <c r="O582" t="s" s="0">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="P582" t="n" s="0">
-        <v>10.0</v>
+        <v>32.0</v>
       </c>
       <c r="Q582" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="R582" t="s" s="0">
-        <v>76</v>
+        <v>39</v>
       </c>
       <c r="S582" t="n" s="0">
         <v>0.0</v>
       </c>
       <c r="T582" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="U582" t="s" s="0">
-        <v>76</v>
+        <v>39</v>
       </c>
       <c r="V582" t="n" s="0">
-        <v>1429.0</v>
+        <v>0.0</v>
       </c>
       <c r="W582" t="s" s="0">
         <v>31</v>
@@ -47924,7 +47924,7 @@
         <v>0.0</v>
       </c>
       <c r="Z582" t="s" s="0">
-        <v>39</v>
+        <v>31</v>
       </c>
     </row>
     <row r="583">
@@ -47971,28 +47971,28 @@
         <v>9.0174073185E10</v>
       </c>
       <c r="O583" t="s" s="0">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="P583" t="n" s="0">
-        <v>32.0</v>
+        <v>10.0</v>
       </c>
       <c r="Q583" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="R583" t="s" s="0">
-        <v>39</v>
+        <v>76</v>
       </c>
       <c r="S583" t="n" s="0">
         <v>0.0</v>
       </c>
       <c r="T583" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="U583" t="s" s="0">
-        <v>39</v>
+        <v>76</v>
       </c>
       <c r="V583" t="n" s="0">
-        <v>0.0</v>
+        <v>1429.0</v>
       </c>
       <c r="W583" t="s" s="0">
         <v>31</v>
@@ -48004,7 +48004,7 @@
         <v>0.0</v>
       </c>
       <c r="Z583" t="s" s="0">
-        <v>31</v>
+        <v>39</v>
       </c>
     </row>
     <row r="584">
@@ -49571,28 +49571,28 @@
         <v>9.0174073185E10</v>
       </c>
       <c r="O603" t="s" s="0">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="P603" t="n" s="0">
-        <v>105.0</v>
+        <v>19.0</v>
       </c>
       <c r="Q603" t="n" s="0">
-        <v>2.0</v>
+        <v>0.0</v>
       </c>
       <c r="R603" t="s" s="0">
-        <v>358</v>
+        <v>39</v>
       </c>
       <c r="S603" t="n" s="0">
         <v>0.0</v>
       </c>
       <c r="T603" t="n" s="0">
-        <v>2.0</v>
+        <v>0.0</v>
       </c>
       <c r="U603" t="s" s="0">
-        <v>358</v>
+        <v>39</v>
       </c>
       <c r="V603" t="n" s="0">
-        <v>858.0</v>
+        <v>0.0</v>
       </c>
       <c r="W603" t="s" s="0">
         <v>31</v>
@@ -49601,10 +49601,10 @@
         <v>38</v>
       </c>
       <c r="Y603" t="n" s="0">
-        <v>48900.0</v>
+        <v>0.0</v>
       </c>
       <c r="Z603" t="s" s="0">
-        <v>359</v>
+        <v>31</v>
       </c>
     </row>
     <row r="604">
@@ -49651,28 +49651,28 @@
         <v>9.0174073185E10</v>
       </c>
       <c r="O604" t="s" s="0">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="P604" t="n" s="0">
-        <v>19.0</v>
+        <v>105.0</v>
       </c>
       <c r="Q604" t="n" s="0">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
       <c r="R604" t="s" s="0">
-        <v>39</v>
+        <v>358</v>
       </c>
       <c r="S604" t="n" s="0">
         <v>0.0</v>
       </c>
       <c r="T604" t="n" s="0">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
       <c r="U604" t="s" s="0">
-        <v>39</v>
+        <v>358</v>
       </c>
       <c r="V604" t="n" s="0">
-        <v>0.0</v>
+        <v>858.0</v>
       </c>
       <c r="W604" t="s" s="0">
         <v>31</v>
@@ -49681,10 +49681,10 @@
         <v>38</v>
       </c>
       <c r="Y604" t="n" s="0">
-        <v>0.0</v>
+        <v>48900.0</v>
       </c>
       <c r="Z604" t="s" s="0">
-        <v>31</v>
+        <v>359</v>
       </c>
     </row>
     <row r="605">
@@ -52931,28 +52931,28 @@
         <v>9.0173710659E10</v>
       </c>
       <c r="O645" t="s" s="0">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="P645" t="n" s="0">
-        <v>39.0</v>
+        <v>356.0</v>
       </c>
       <c r="Q645" t="n" s="0">
-        <v>1.0</v>
+        <v>5.0</v>
       </c>
       <c r="R645" t="s" s="0">
-        <v>157</v>
+        <v>376</v>
       </c>
       <c r="S645" t="n" s="0">
         <v>0.0</v>
       </c>
       <c r="T645" t="n" s="0">
-        <v>1.0</v>
+        <v>5.0</v>
       </c>
       <c r="U645" t="s" s="0">
-        <v>157</v>
+        <v>376</v>
       </c>
       <c r="V645" t="n" s="0">
-        <v>2082.0</v>
+        <v>1739.0</v>
       </c>
       <c r="W645" t="s" s="0">
         <v>31</v>
@@ -53011,28 +53011,28 @@
         <v>9.0173710659E10</v>
       </c>
       <c r="O646" t="s" s="0">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="P646" t="n" s="0">
-        <v>356.0</v>
+        <v>39.0</v>
       </c>
       <c r="Q646" t="n" s="0">
-        <v>5.0</v>
+        <v>1.0</v>
       </c>
       <c r="R646" t="s" s="0">
-        <v>376</v>
+        <v>157</v>
       </c>
       <c r="S646" t="n" s="0">
         <v>0.0</v>
       </c>
       <c r="T646" t="n" s="0">
-        <v>5.0</v>
+        <v>1.0</v>
       </c>
       <c r="U646" t="s" s="0">
-        <v>376</v>
+        <v>157</v>
       </c>
       <c r="V646" t="n" s="0">
-        <v>1739.0</v>
+        <v>2082.0</v>
       </c>
       <c r="W646" t="s" s="0">
         <v>31</v>
@@ -53349,7 +53349,7 @@
         <v>6.0</v>
       </c>
       <c r="U650" t="s" s="0">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="V650" t="n" s="0">
         <v>154.0</v>
@@ -53491,28 +53491,28 @@
         <v>9.0173710659E10</v>
       </c>
       <c r="O652" t="s" s="0">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="P652" t="n" s="0">
-        <v>33.0</v>
+        <v>299.0</v>
       </c>
       <c r="Q652" t="n" s="0">
-        <v>0.0</v>
+        <v>5.0</v>
       </c>
       <c r="R652" t="s" s="0">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="S652" t="n" s="0">
         <v>0.0</v>
       </c>
       <c r="T652" t="n" s="0">
-        <v>0.0</v>
+        <v>5.0</v>
       </c>
       <c r="U652" t="s" s="0">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="V652" t="n" s="0">
-        <v>0.0</v>
+        <v>4853.0</v>
       </c>
       <c r="W652" t="s" s="0">
         <v>31</v>
@@ -53524,7 +53524,7 @@
         <v>0.0</v>
       </c>
       <c r="Z652" t="s" s="0">
-        <v>31</v>
+        <v>39</v>
       </c>
     </row>
     <row r="653">
@@ -53571,28 +53571,28 @@
         <v>9.0173710659E10</v>
       </c>
       <c r="O653" t="s" s="0">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="P653" t="n" s="0">
-        <v>299.0</v>
+        <v>33.0</v>
       </c>
       <c r="Q653" t="n" s="0">
-        <v>5.0</v>
+        <v>0.0</v>
       </c>
       <c r="R653" t="s" s="0">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="S653" t="n" s="0">
         <v>0.0</v>
       </c>
       <c r="T653" t="n" s="0">
-        <v>5.0</v>
+        <v>0.0</v>
       </c>
       <c r="U653" t="s" s="0">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="V653" t="n" s="0">
-        <v>4853.0</v>
+        <v>0.0</v>
       </c>
       <c r="W653" t="s" s="0">
         <v>31</v>
@@ -53604,7 +53604,7 @@
         <v>0.0</v>
       </c>
       <c r="Z653" t="s" s="0">
-        <v>39</v>
+        <v>31</v>
       </c>
     </row>
     <row r="654">
@@ -53811,10 +53811,10 @@
         <v>0.0</v>
       </c>
       <c r="O656" t="s" s="0">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="P656" t="n" s="0">
-        <v>8.0</v>
+        <v>44.0</v>
       </c>
       <c r="Q656" t="n" s="0">
         <v>0.0</v>
@@ -53823,16 +53823,16 @@
         <v>39</v>
       </c>
       <c r="S656" t="n" s="0">
-        <v>2.0</v>
+        <v>7.0</v>
       </c>
       <c r="T656" t="n" s="0">
-        <v>2.0</v>
+        <v>7.0</v>
       </c>
       <c r="U656" t="s" s="0">
-        <v>80</v>
+        <v>378</v>
       </c>
       <c r="V656" t="n" s="0">
-        <v>11.0</v>
+        <v>231.0</v>
       </c>
       <c r="W656" t="s" s="0">
         <v>31</v>
@@ -53891,10 +53891,10 @@
         <v>0.0</v>
       </c>
       <c r="O657" t="s" s="0">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="P657" t="n" s="0">
-        <v>44.0</v>
+        <v>8.0</v>
       </c>
       <c r="Q657" t="n" s="0">
         <v>0.0</v>
@@ -53903,16 +53903,16 @@
         <v>39</v>
       </c>
       <c r="S657" t="n" s="0">
-        <v>7.0</v>
+        <v>2.0</v>
       </c>
       <c r="T657" t="n" s="0">
-        <v>7.0</v>
+        <v>2.0</v>
       </c>
       <c r="U657" t="s" s="0">
-        <v>378</v>
+        <v>80</v>
       </c>
       <c r="V657" t="n" s="0">
-        <v>231.0</v>
+        <v>11.0</v>
       </c>
       <c r="W657" t="s" s="0">
         <v>31</v>
@@ -54460,7 +54460,7 @@
         <v>1.0</v>
       </c>
       <c r="R664" t="s" s="0">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="S664" t="n" s="0">
         <v>6.0</v>
@@ -54931,10 +54931,10 @@
         <v>0.0</v>
       </c>
       <c r="O670" t="s" s="0">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="P670" t="n" s="0">
-        <v>24.0</v>
+        <v>146.0</v>
       </c>
       <c r="Q670" t="n" s="0">
         <v>0.0</v>
@@ -54943,16 +54943,16 @@
         <v>39</v>
       </c>
       <c r="S670" t="n" s="0">
-        <v>9.0</v>
+        <v>17.0</v>
       </c>
       <c r="T670" t="n" s="0">
-        <v>9.0</v>
+        <v>17.0</v>
       </c>
       <c r="U670" t="s" s="0">
-        <v>251</v>
+        <v>381</v>
       </c>
       <c r="V670" t="n" s="0">
-        <v>112.0</v>
+        <v>962.0</v>
       </c>
       <c r="W670" t="s" s="0">
         <v>31</v>
@@ -55011,10 +55011,10 @@
         <v>0.0</v>
       </c>
       <c r="O671" t="s" s="0">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="P671" t="n" s="0">
-        <v>146.0</v>
+        <v>24.0</v>
       </c>
       <c r="Q671" t="n" s="0">
         <v>0.0</v>
@@ -55023,16 +55023,16 @@
         <v>39</v>
       </c>
       <c r="S671" t="n" s="0">
-        <v>17.0</v>
+        <v>9.0</v>
       </c>
       <c r="T671" t="n" s="0">
-        <v>17.0</v>
+        <v>9.0</v>
       </c>
       <c r="U671" t="s" s="0">
-        <v>381</v>
+        <v>251</v>
       </c>
       <c r="V671" t="n" s="0">
-        <v>962.0</v>
+        <v>112.0</v>
       </c>
       <c r="W671" t="s" s="0">
         <v>31</v>
@@ -56051,28 +56051,28 @@
         <v>9.157937742E10</v>
       </c>
       <c r="O684" t="s" s="0">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="P684" t="n" s="0">
-        <v>129.0</v>
+        <v>171.0</v>
       </c>
       <c r="Q684" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="R684" t="s" s="0">
-        <v>39</v>
+        <v>391</v>
       </c>
       <c r="S684" t="n" s="0">
         <v>0.0</v>
       </c>
       <c r="T684" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="U684" t="s" s="0">
-        <v>39</v>
+        <v>391</v>
       </c>
       <c r="V684" t="n" s="0">
-        <v>0.0</v>
+        <v>2692.0</v>
       </c>
       <c r="W684" t="s" s="0">
         <v>31</v>
@@ -56084,7 +56084,7 @@
         <v>0.0</v>
       </c>
       <c r="Z684" t="s" s="0">
-        <v>31</v>
+        <v>39</v>
       </c>
     </row>
     <row r="685">
@@ -56131,28 +56131,28 @@
         <v>9.157937742E10</v>
       </c>
       <c r="O685" t="s" s="0">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="P685" t="n" s="0">
-        <v>171.0</v>
+        <v>129.0</v>
       </c>
       <c r="Q685" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="R685" t="s" s="0">
-        <v>391</v>
+        <v>39</v>
       </c>
       <c r="S685" t="n" s="0">
         <v>0.0</v>
       </c>
       <c r="T685" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="U685" t="s" s="0">
-        <v>391</v>
+        <v>39</v>
       </c>
       <c r="V685" t="n" s="0">
-        <v>2692.0</v>
+        <v>0.0</v>
       </c>
       <c r="W685" t="s" s="0">
         <v>31</v>
@@ -56164,7 +56164,7 @@
         <v>0.0</v>
       </c>
       <c r="Z685" t="s" s="0">
-        <v>39</v>
+        <v>31</v>
       </c>
     </row>
     <row r="686">
@@ -57331,28 +57331,28 @@
         <v>9.157937742E10</v>
       </c>
       <c r="O700" t="s" s="0">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="P700" t="n" s="0">
-        <v>26.0</v>
+        <v>25.0</v>
       </c>
       <c r="Q700" t="n" s="0">
-        <v>2.0</v>
+        <v>0.0</v>
       </c>
       <c r="R700" t="s" s="0">
-        <v>263</v>
+        <v>39</v>
       </c>
       <c r="S700" t="n" s="0">
         <v>0.0</v>
       </c>
       <c r="T700" t="n" s="0">
-        <v>2.0</v>
+        <v>0.0</v>
       </c>
       <c r="U700" t="s" s="0">
-        <v>263</v>
+        <v>39</v>
       </c>
       <c r="V700" t="n" s="0">
-        <v>1310.0</v>
+        <v>0.0</v>
       </c>
       <c r="W700" t="s" s="0">
         <v>31</v>
@@ -57364,7 +57364,7 @@
         <v>0.0</v>
       </c>
       <c r="Z700" t="s" s="0">
-        <v>39</v>
+        <v>31</v>
       </c>
     </row>
     <row r="701">
@@ -57411,28 +57411,28 @@
         <v>9.157937742E10</v>
       </c>
       <c r="O701" t="s" s="0">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="P701" t="n" s="0">
-        <v>25.0</v>
+        <v>26.0</v>
       </c>
       <c r="Q701" t="n" s="0">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
       <c r="R701" t="s" s="0">
-        <v>39</v>
+        <v>263</v>
       </c>
       <c r="S701" t="n" s="0">
         <v>0.0</v>
       </c>
       <c r="T701" t="n" s="0">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
       <c r="U701" t="s" s="0">
-        <v>39</v>
+        <v>263</v>
       </c>
       <c r="V701" t="n" s="0">
-        <v>0.0</v>
+        <v>1310.0</v>
       </c>
       <c r="W701" t="s" s="0">
         <v>31</v>
@@ -57444,7 +57444,7 @@
         <v>0.0</v>
       </c>
       <c r="Z701" t="s" s="0">
-        <v>31</v>
+        <v>39</v>
       </c>
     </row>
     <row r="702">
@@ -57971,10 +57971,10 @@
         <v>9.157937742E10</v>
       </c>
       <c r="O708" t="s" s="0">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="P708" t="n" s="0">
-        <v>42.0</v>
+        <v>23.0</v>
       </c>
       <c r="Q708" t="n" s="0">
         <v>0.0</v>
@@ -58051,10 +58051,10 @@
         <v>9.157937742E10</v>
       </c>
       <c r="O709" t="s" s="0">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="P709" t="n" s="0">
-        <v>23.0</v>
+        <v>42.0</v>
       </c>
       <c r="Q709" t="n" s="0">
         <v>0.0</v>
@@ -59260,7 +59260,7 @@
         <v>2.0</v>
       </c>
       <c r="R724" t="s" s="0">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="S724" t="n" s="0">
         <v>0.0</v>
@@ -59269,7 +59269,7 @@
         <v>2.0</v>
       </c>
       <c r="U724" t="s" s="0">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="V724" t="n" s="0">
         <v>932.0</v>
@@ -63580,7 +63580,7 @@
         <v>19.0</v>
       </c>
       <c r="R778" t="s" s="0">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="S778" t="n" s="0">
         <v>0.0</v>
@@ -63589,7 +63589,7 @@
         <v>19.0</v>
       </c>
       <c r="U778" t="s" s="0">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="V778" t="n" s="0">
         <v>6614.0</v>
@@ -64051,28 +64051,28 @@
         <v>9.1134901349E10</v>
       </c>
       <c r="O784" t="s" s="0">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="P784" t="n" s="0">
-        <v>0.0</v>
+        <v>373.0</v>
       </c>
       <c r="Q784" t="n" s="0">
-        <v>7.0</v>
+        <v>13.0</v>
       </c>
       <c r="R784" t="s" s="0">
-        <v>39</v>
+        <v>430</v>
       </c>
       <c r="S784" t="n" s="0">
         <v>0.0</v>
       </c>
       <c r="T784" t="n" s="0">
-        <v>7.0</v>
+        <v>13.0</v>
       </c>
       <c r="U784" t="s" s="0">
-        <v>31</v>
+        <v>430</v>
       </c>
       <c r="V784" t="n" s="0">
-        <v>0.0</v>
+        <v>3813.0</v>
       </c>
       <c r="W784" t="s" s="0">
         <v>31</v>
@@ -64084,7 +64084,7 @@
         <v>0.0</v>
       </c>
       <c r="Z784" t="s" s="0">
-        <v>31</v>
+        <v>39</v>
       </c>
     </row>
     <row r="785">
@@ -64131,28 +64131,28 @@
         <v>9.1134901349E10</v>
       </c>
       <c r="O785" t="s" s="0">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="P785" t="n" s="0">
-        <v>373.0</v>
+        <v>0.0</v>
       </c>
       <c r="Q785" t="n" s="0">
-        <v>13.0</v>
+        <v>7.0</v>
       </c>
       <c r="R785" t="s" s="0">
-        <v>430</v>
+        <v>39</v>
       </c>
       <c r="S785" t="n" s="0">
         <v>0.0</v>
       </c>
       <c r="T785" t="n" s="0">
-        <v>13.0</v>
+        <v>7.0</v>
       </c>
       <c r="U785" t="s" s="0">
-        <v>430</v>
+        <v>31</v>
       </c>
       <c r="V785" t="n" s="0">
-        <v>3813.0</v>
+        <v>0.0</v>
       </c>
       <c r="W785" t="s" s="0">
         <v>31</v>
@@ -64164,7 +64164,7 @@
         <v>0.0</v>
       </c>
       <c r="Z785" t="s" s="0">
-        <v>39</v>
+        <v>31</v>
       </c>
     </row>
     <row r="786">

</xml_diff>